<commit_message>
fix: colores CheckRates + canastas Top5 RatesNoDispo + guía editorial unificada
</commit_message>
<xml_diff>
--- a/checkrates/week-16/Analisis/Analisis_Checkrates_7d.xlsx
+++ b/checkrates/week-16/Analisis/Analisis_Checkrates_7d.xlsx
@@ -34,7 +34,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -83,8 +83,20 @@
       <color rgb="0014304A"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00F8F4EC"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00F8F4EC"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -139,6 +151,26 @@
         <bgColor rgb="00E8F3F8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00161616"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EA0074"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005C469C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004FC3F4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="6">
     <border>
@@ -177,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -229,6 +261,27 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -603,12 +656,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  FICHA TÉCNICA · Supply CheckRates · Week 16</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -901,7 +955,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Connectivity Issue · Monetization Failure · Quick Win · Low Priority</t>
+          <t>Connectivity Issue · Sin Conversión · Quick Win · Low Priority</t>
         </is>
       </c>
     </row>
@@ -947,12 +1001,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  PLAN DE ACCIÓN · Quick Wins / Mid-term / Estratégico</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -1089,7 +1144,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Diagnóstico de 856 hoteles Monetization Failure</t>
+          <t>Diagnóstico de 856 hoteles Sin Conversión</t>
         </is>
       </c>
       <c r="C7" s="17" t="inlineStr">
@@ -1333,12 +1388,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  CANASTA B2C · HOTELES CRÍTICOS · Top 20 · Eficacia + Conv Rate</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -1407,7 +1463,7 @@
       <c r="G4" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1439,7 +1495,7 @@
       <c r="G5" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1471,7 +1527,7 @@
       <c r="G6" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1503,7 +1559,7 @@
       <c r="G7" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1535,7 +1591,7 @@
       <c r="G8" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1567,7 +1623,7 @@
       <c r="G9" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1599,7 +1655,7 @@
       <c r="G10" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1631,7 +1687,7 @@
       <c r="G11" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1663,7 +1719,7 @@
       <c r="G12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H12" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1695,7 +1751,7 @@
       <c r="G13" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1727,7 +1783,7 @@
       <c r="G14" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H14" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1759,7 +1815,7 @@
       <c r="G15" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1791,7 +1847,7 @@
       <c r="G16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H16" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1823,7 +1879,7 @@
       <c r="G17" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1855,7 +1911,7 @@
       <c r="G18" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H18" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1887,7 +1943,7 @@
       <c r="G19" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1951,7 +2007,7 @@
       <c r="G21" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="H21" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -1983,7 +2039,7 @@
       <c r="G22" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -2015,7 +2071,7 @@
       <c r="G23" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="H23" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -2049,12 +2105,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  CANASTA B2C · BAJO RENDIMIENTO · Top 20 · %Errors ≥ 5.3% y Bookings &gt; 0</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -2725,12 +2782,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  CANASTA B2B (OP) · HOTELES CRÍTICOS · Top 20 · Eficacia + Conv Rate</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2799,7 +2857,7 @@
       <c r="G4" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -2831,7 +2889,7 @@
       <c r="G5" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -2863,7 +2921,7 @@
       <c r="G6" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -2895,7 +2953,7 @@
       <c r="G7" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="H7" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -2927,7 +2985,7 @@
       <c r="G8" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -2959,7 +3017,7 @@
       <c r="G9" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -2991,7 +3049,7 @@
       <c r="G10" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -3023,7 +3081,7 @@
       <c r="G11" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="H11" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -3087,7 +3145,7 @@
       <c r="G13" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="H13" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -3119,7 +3177,7 @@
       <c r="G14" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="H14" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -3151,7 +3209,7 @@
       <c r="G15" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -3247,7 +3305,7 @@
       <c r="G18" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H18" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -3311,7 +3369,7 @@
       <c r="G20" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H20" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -3441,12 +3499,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  CANASTA B2B (OP) · BAJO RENDIMIENTO · Top 20 · %Errors ≥ 5.3% y Bookings &gt; 0</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -4117,12 +4176,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  CANASTA CUG (UOP) · HOTELES CRÍTICOS · Top 20 · Eficacia + Conv Rate</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -4255,9 +4315,9 @@
       <c r="G6" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Monetization Failure</t>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>Sin Conversión</t>
         </is>
       </c>
     </row>
@@ -4351,7 +4411,7 @@
       <c r="G9" s="11" t="n">
         <v>0.002607561929595828</v>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="24" t="inlineStr">
         <is>
           <t>Quick Win</t>
         </is>
@@ -4383,7 +4443,7 @@
       <c r="G10" s="11" t="n">
         <v>0.004909983633387889</v>
       </c>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="H10" s="24" t="inlineStr">
         <is>
           <t>Quick Win</t>
         </is>
@@ -4511,9 +4571,9 @@
       <c r="G14" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>Monetization Failure</t>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>Sin Conversión</t>
         </is>
       </c>
     </row>
@@ -4543,7 +4603,7 @@
       <c r="G15" s="11" t="n">
         <v>0.003853564547206166</v>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H15" s="24" t="inlineStr">
         <is>
           <t>Quick Win</t>
         </is>
@@ -4575,7 +4635,7 @@
       <c r="G16" s="11" t="n">
         <v>0.01120448179271709</v>
       </c>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="H16" s="24" t="inlineStr">
         <is>
           <t>Quick Win</t>
         </is>
@@ -4607,7 +4667,7 @@
       <c r="G17" s="11" t="n">
         <v>0.01048689138576779</v>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H17" s="24" t="inlineStr">
         <is>
           <t>Quick Win</t>
         </is>
@@ -4671,7 +4731,7 @@
       <c r="G19" s="11" t="n">
         <v>0.001464128843338214</v>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="24" t="inlineStr">
         <is>
           <t>Quick Win</t>
         </is>
@@ -4703,7 +4763,7 @@
       <c r="G20" s="11" t="n">
         <v>0.0006939625260235947</v>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H20" s="24" t="inlineStr">
         <is>
           <t>Quick Win</t>
         </is>
@@ -4735,7 +4795,7 @@
       <c r="G21" s="11" t="n">
         <v>0.005701254275940707</v>
       </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="H21" s="24" t="inlineStr">
         <is>
           <t>Quick Win</t>
         </is>
@@ -4767,7 +4827,7 @@
       <c r="G22" s="11" t="n">
         <v>0.00196969696969697</v>
       </c>
-      <c r="H22" s="6" t="inlineStr">
+      <c r="H22" s="24" t="inlineStr">
         <is>
           <t>Quick Win</t>
         </is>
@@ -4833,12 +4893,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  CANASTA CUG (UOP) · BAJO RENDIMIENTO · Top 20 · %Errors ≥ 5.3% y Bookings &gt; 0</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -5506,12 +5567,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEVERITY · EFICACIA · Distribución Muestra HTS · P80</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -5702,12 +5764,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEVERITY · CONV RATE · Distribución Muestra HTS · P80</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -5901,12 +5964,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  HOTELES CRÍTICOS · Top 20 · Eficacia + Conv Rate · CheckRates ≥1K</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -5975,7 +6039,7 @@
       <c r="G4" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -6007,7 +6071,7 @@
       <c r="G5" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -6103,7 +6167,7 @@
       <c r="G8" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="6" t="inlineStr">
+      <c r="H8" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -6135,7 +6199,7 @@
       <c r="G9" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H9" s="22" t="inlineStr">
         <is>
           <t>Connectivity Issue</t>
         </is>
@@ -6295,9 +6359,9 @@
       <c r="G14" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>Monetization Failure</t>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>Sin Conversión</t>
         </is>
       </c>
     </row>
@@ -6455,7 +6519,7 @@
       <c r="G19" s="11" t="n">
         <v>0.0003918495297805642</v>
       </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="H19" s="24" t="inlineStr">
         <is>
           <t>Quick Win</t>
         </is>
@@ -6583,9 +6647,9 @@
       <c r="G23" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>Monetization Failure</t>
+      <c r="H23" s="23" t="inlineStr">
+        <is>
+          <t>Sin Conversión</t>
         </is>
       </c>
     </row>
@@ -6617,12 +6681,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  BAJO RENDIMIENTO · Top 20 · %Errors ≥ 5.3% y Bookings &gt; 0</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -7293,12 +7358,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  POR CORPORATIVO · Top 20 · ordenado por Conv Rate ↑ · ≥5 hoteles HTS</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -7930,12 +7996,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEVERITY POR CORPORATIVO · EFICACIA · Top 20</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -8632,12 +8699,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  SEVERITY POR CORPORATIVO · CONV RATE · Top 20</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -9332,12 +9400,13 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+      <c r="A1" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  MENOR CONV RATE · Top 20 · Bookings &gt; 0 · CheckRates ≥ P50 Muestra</t>
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="15" t="inlineStr">
         <is>

</xml_diff>